<commit_message>
Transfer fix: multi-leg AddFundings body + zero-lender guard
</commit_message>
<xml_diff>
--- a/dist/loan-history-replay-bundle/test-addfunding-sample.xlsx
+++ b/dist/loan-history-replay-bundle/test-addfunding-sample.xlsx
@@ -454,7 +454,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>REPLACE_WITH_REAL_LENDER_CODE</t>
+          <t>REPLACE_WITH_REAL_LENDER_ACCOUNT</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -463,7 +463,7 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>0.01</v>
+        <v>100</v>
       </c>
       <c r="E2" s="1" t="n">
         <v>45901</v>

</xml_diff>